<commit_message>
Commit <Prompt for second part>
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ALTFEST_DA_User1\Documents\UiPath\Altfest_TaxReturnP1\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82211B26-19B5-4F75-8676-33179EC555FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AF88CB8-9200-4C69-9D66-31EDCC16C6C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -243,9 +243,6 @@
     <t>Stores the login URL used to access Practifi for Altfest.</t>
   </si>
   <si>
-    <t>C:\Users\ALTFEST_DA_User2\Documents\Altfest\Output\[PreviousYear] Tax Returns Received [CurrentDate].xlsx</t>
-  </si>
-  <si>
     <t>MaxApiRetry</t>
   </si>
   <si>
@@ -291,10 +288,13 @@
     <t>MasterFilePath1</t>
   </si>
   <si>
-    <t>C:\Users\ALTFEST_DA_User1\Documents\TaxReturnPt1\Output\2025 Tax Returns Received 07.31.26.xlsx</t>
-  </si>
-  <si>
-    <t>C:\Users\ALTFEST_DA_User1\Documents\TaxReturnPt1\TaxReturnOutput_Template.xlsx</t>
+    <t>[DocumentFolderPath]\TaxReturnPt1\TaxReturnOutput_Template.xlsx</t>
+  </si>
+  <si>
+    <t>[DocumentFolderPath]\TaxReturnPt1\Output\2025 Tax Returns Received 07.31.26.xlsx</t>
+  </si>
+  <si>
+    <t>[DocumentFolderPath]\TaxReturnPt1\Output\[PreviousYear] Tax Returns Received [CurrentDate].xlsx</t>
   </si>
 </sst>
 </file>
@@ -362,7 +362,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -378,8 +378,6 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1964,12 +1962,12 @@
         <v>46</v>
       </c>
     </row>
-    <row r="20" spans="1:3" ht="14.25" customHeight="1">
-      <c r="A20" s="2" t="s">
+    <row r="20" spans="1:3" s="8" customFormat="1" ht="14.25" customHeight="1">
+      <c r="A20" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="B20" t="s">
-        <v>68</v>
+      <c r="B20" s="8" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="21" spans="1:3" ht="14.25" customHeight="1">
@@ -1985,7 +1983,7 @@
         <v>51</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="23" spans="1:3" ht="14.25" customHeight="1">
@@ -2001,15 +1999,15 @@
         <v>54</v>
       </c>
       <c r="B24" s="8" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" ht="14.25" customHeight="1">
+      <c r="A25" s="2" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="25" spans="1:3" s="10" customFormat="1" ht="14.25" customHeight="1">
-      <c r="A25" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="B25" s="10" t="s">
-        <v>70</v>
+      <c r="B25" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="26" spans="1:3" ht="14.25" customHeight="1">
@@ -2038,7 +2036,7 @@
     </row>
     <row r="29" spans="1:3" ht="14.25" customHeight="1">
       <c r="A29" s="2" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B29">
         <v>3</v>
@@ -2046,31 +2044,31 @@
     </row>
     <row r="30" spans="1:3" ht="14.25" customHeight="1">
       <c r="A30" s="2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B30" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="31" spans="1:3" ht="14.25" customHeight="1">
       <c r="A31" t="s">
+        <v>75</v>
+      </c>
+      <c r="B31" t="s">
         <v>76</v>
-      </c>
-      <c r="B31" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="32" spans="1:3" ht="14.25" customHeight="1">
       <c r="A32" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="33" spans="1:2" s="8" customFormat="1" ht="14.25" customHeight="1">
       <c r="A33" s="7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B33" s="7" t="s">
         <v>84</v>
@@ -2078,7 +2076,7 @@
     </row>
     <row r="34" spans="1:2" ht="14.25" customHeight="1">
       <c r="A34" s="2" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B34">
         <v>3</v>
@@ -3117,7 +3115,7 @@
         <v>44</v>
       </c>
       <c r="D3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1">
@@ -3131,7 +3129,7 @@
         <v>44</v>
       </c>
       <c r="D4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="5" spans="1:26" ht="14.25" customHeight="1">
@@ -3145,7 +3143,7 @@
         <v>44</v>
       </c>
       <c r="D5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6" spans="1:26" ht="14.25" customHeight="1">
@@ -3164,10 +3162,10 @@
     </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1">
       <c r="A7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B7" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C7" t="s">
         <v>44</v>

</xml_diff>